<commit_message>
fin resultats all data
</commit_message>
<xml_diff>
--- a/results_all_data/describ_graphs_0.95.xlsx
+++ b/results_all_data/describ_graphs_0.95.xlsx
@@ -395,10 +395,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>6.22222222222222</v>
+        <v>6.38461538461539</v>
       </c>
       <c r="C2" t="n">
-        <v>0.239316239316239</v>
+        <v>0.255384615384615</v>
       </c>
     </row>
     <row r="3">
@@ -406,10 +406,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>7.40740740740741</v>
+        <v>6.69230769230769</v>
       </c>
       <c r="C3" t="n">
-        <v>0.284900284900285</v>
+        <v>0.267692307692308</v>
       </c>
     </row>
     <row r="4">
@@ -417,10 +417,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>7.25925925925926</v>
+        <v>6.76923076923077</v>
       </c>
       <c r="C4" t="n">
-        <v>0.279202279202279</v>
+        <v>0.270769230769231</v>
       </c>
     </row>
     <row r="5">
@@ -428,10 +428,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>7.62962962962963</v>
+        <v>6.84615384615385</v>
       </c>
       <c r="C5" t="n">
-        <v>0.293447293447293</v>
+        <v>0.273846153846154</v>
       </c>
     </row>
     <row r="6">
@@ -439,10 +439,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>7.85185185185185</v>
+        <v>7</v>
       </c>
       <c r="C6" t="n">
-        <v>0.301994301994302</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="7">
@@ -450,10 +450,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>1.92592592592593</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0740740740740741</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="8">
@@ -461,10 +461,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>2.37037037037037</v>
+        <v>1.92307692307692</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0911680911680912</v>
+        <v>0.0769230769230769</v>
       </c>
     </row>
     <row r="9">
@@ -472,10 +472,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>2.2962962962963</v>
+        <v>1.76923076923077</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0883190883190883</v>
+        <v>0.0707692307692308</v>
       </c>
     </row>
     <row r="10">
@@ -483,10 +483,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>2.51851851851852</v>
+        <v>2.23076923076923</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0968660968660969</v>
+        <v>0.0892307692307692</v>
       </c>
     </row>
     <row r="11">
@@ -494,10 +494,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>2.59259259259259</v>
+        <v>2.07692307692308</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0997150997150997</v>
+        <v>0.0830769230769231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>